<commit_message>
Create new question workbook
</commit_message>
<xml_diff>
--- a/KT_Session_Question_Review/00_Drafts/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
+++ b/KT_Session_Question_Review/00_Drafts/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lambert/Documents/Projects/SHRSS/SHRSS_Knowledge_Transfer/KT_Session_Question_Review/00_Drafts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7981DDE9-4CB0-344F-8565-31BE95D47311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176D4119-FECA-704C-91BA-800245DDB041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="780" windowWidth="24040" windowHeight="21580" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="780" windowWidth="24040" windowHeight="21580" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jobs" sheetId="1" r:id="rId1"/>
@@ -25,13 +25,15 @@
     <sheet name="Media" sheetId="10" r:id="rId10"/>
     <sheet name="Page_Templates" sheetId="11" r:id="rId11"/>
     <sheet name="Navigation_and_Data_Display" sheetId="12" r:id="rId12"/>
+    <sheet name="LOB_Specific" sheetId="13" r:id="rId13"/>
+    <sheet name="Sheet4" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1678" uniqueCount="689">
   <si>
     <t>Status</t>
   </si>
@@ -1690,13 +1692,421 @@
   </si>
   <si>
     <t>How should authors ensure tables remain readable on mobile devices?</t>
+  </si>
+  <si>
+    <t>Is the location that appears in the delivery widget coming from DPLT?</t>
+  </si>
+  <si>
+    <t>Why does the disclaimer text look visually disconnected from the content when the widget is not placed in a container with the production background styling?</t>
+  </si>
+  <si>
+    <t>Can we control which locations appear in the “Reserve a Table” dropdown list (for example only US locations or only specific locations for a promotion)?</t>
+  </si>
+  <si>
+    <t>Is the “Reserve Table” experience fragment created inside every cafe folder?</t>
+  </si>
+  <si>
+    <t>Why is the button appearing purple in the example?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Rick Lyon </t>
+  </si>
+  <si>
+    <t>Are there safeguards for third-party reservation widgets if the embed code is very large or poorly styled (too wide or too tall)?</t>
+  </si>
+  <si>
+    <t>If a cafe uses a reservation widget other than OpenTable, will that same widget appear in the Reserve Table modal?</t>
+  </si>
+  <si>
+    <t>For a location like Porto that uses a different reservation system, how would that embed be handled in AEM?</t>
+  </si>
+  <si>
+    <t>How should phone numbers be entered so the tel: link works correctly while still displaying formatted characters like dashes?</t>
+  </si>
+  <si>
+    <t>If fields like phone number or email are blank, will the associated icons still display?</t>
+  </si>
+  <si>
+    <t>Where do we link the menu PDFs within the dining reservation component?</t>
+  </si>
+  <si>
+    <t>Do we have recommended image dimensions for the images used in the microsite card placements?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Lisa Cardia @Don Middlebrook </t>
+  </si>
+  <si>
+    <t>Can the title color be changed in the Messi Experience component?</t>
+  </si>
+  <si>
+    <t>Why does Button 2 allow opening a modal but Button 1 does not?</t>
+  </si>
+  <si>
+    <t>On mobile, why are the titles and text left-aligned while the buttons appear centered?</t>
+  </si>
+  <si>
+    <t>How does the component behave if location services are disabled in the browser?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Mayte Eme </t>
+  </si>
+  <si>
+    <t>How frequently does AEM refresh location data coming from DPLT content fragments?</t>
+  </si>
+  <si>
+    <t>If a delivery partner URL is removed from a location content fragment, how quickly does it stop appearing in the widget?</t>
+  </si>
+  <si>
+    <t>Is there any sorting logic applied to the delivery partner dropdown (priority order, alphabetical, etc.)?</t>
+  </si>
+  <si>
+    <t>What happens if a cafe does not have a Reserve Table experience fragment created?</t>
+  </si>
+  <si>
+    <t>Is there any validation to prevent duplicate experience fragment names across cafes?</t>
+  </si>
+  <si>
+    <t>Does the system require publishing both the experience fragment and the page for the modal to work?</t>
+  </si>
+  <si>
+    <t>Are there recommended styling constraints for embedded widgets inside the modal?</t>
+  </si>
+  <si>
+    <t>Is there a maximum number of menus that should be added before usability becomes difficult?</t>
+  </si>
+  <si>
+    <t>If a social platform is deprecated or removed (like X/Twitter), how is the icon list updated across existing pages?</t>
+  </si>
+  <si>
+    <t>Are generic lists environment specific, or are they shared across dev, stage, and production?</t>
+  </si>
+  <si>
+    <t>Is there version control or auditing for changes made to generic lists?</t>
+  </si>
+  <si>
+    <t>Which of the components shown today are intended to be reusable across other sites (hotels, corporate, etc.)?</t>
+  </si>
+  <si>
+    <t>Are there components that were built specifically for one campaign or microsite and should not be reused? and why?</t>
+  </si>
+  <si>
+    <t>How should authors validate that newly added delivery partner links work correctly before publishing?</t>
+  </si>
+  <si>
+    <t>Can authors temporarily disable a social icon without deleting the configuration?</t>
+  </si>
+  <si>
+    <t>How should authors handle situations where a location does not have social media profiles?</t>
+  </si>
+  <si>
+    <t>How can authors verify that the Reserve Table experience fragment was configured correctly for a new location?</t>
+  </si>
+  <si>
+    <t>What troubleshooting steps should authors follow if the Reserve Table modal displays empty content?</t>
+  </si>
+  <si>
+    <t>Which components demonstrated in this session are considered core reusable components versus campaign-specific components?</t>
+  </si>
+  <si>
+    <t>Are delivery partner links marked with appropriate link attributes (nofollow, sponsored, etc.)?</t>
+  </si>
+  <si>
+    <t>Does the delivery widget generate crawlable links, or are they hidden behind JavaScript interactions?</t>
+  </si>
+  <si>
+    <t>Do reservation links include tracking parameters or canonical link considerations?</t>
+  </si>
+  <si>
+    <t>do menu links include structured data for restaurant menus?</t>
+  </si>
+  <si>
+    <t>Does the microsite template allow authors to configure meta titles, descriptions, and canonical tags?</t>
+  </si>
+  <si>
+    <t>Are anchor links in the microsite navigation considered SEO-friendly internal links?</t>
+  </si>
+  <si>
+    <t>Could parallax animations affect content indexing or accessibility for search engines?</t>
+  </si>
+  <si>
+    <t>Is the content within animated containers visible in the HTML DOM before animations trigger?</t>
+  </si>
+  <si>
+    <t>Are clicks on delivery partner links tracked as separate analytics events?</t>
+  </si>
+  <si>
+    <t>Can analytics distinguish between different delivery partners selected by users?</t>
+  </si>
+  <si>
+    <t>Can analytics identify which reservation platform generated the interaction?</t>
+  </si>
+  <si>
+    <t>Can we track which cafe location users select within the modal dropdown?</t>
+  </si>
+  <si>
+    <t>Do we have recommended image dimensions for the images used in the Delivery widget?</t>
+  </si>
+  <si>
+    <t>Why is the text not Rich Text for the Delivery Widget?</t>
+  </si>
+  <si>
+    <t>Can we update the Menu Asset Path folder to start with Assets instead of sites? Authors cannot add menus.</t>
+  </si>
+  <si>
+    <t>Do we have recommended image dimensions for the images used in the Messi Experience?</t>
+  </si>
+  <si>
+    <t>Do we have recommended image dimensions for the images used in the Microsite Banner?</t>
+  </si>
+  <si>
+    <t>What does ‘Copy Link to’ do in Microsite Banner?</t>
+  </si>
+  <si>
+    <t>What size logo is necessary for Microsite Navigation?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Button - Allows you to display an icon inside the button (availability depends on your CMS configuration). What is an example of this icon? Can we use fontawesome? </t>
+  </si>
+  <si>
+    <t>Accordion - Why does the containers for 1 &amp; 2 automatically set to no width, but as soon as you add item 3, it’s set to content area and then an author has to adjust items 1, 2 and 3?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabs Cards Filter - What is paragraph system – HTL? </t>
+  </si>
+  <si>
+    <t>Card Carousel - Why does the Panel Selector not work for this component? Can we look at all components with Panel Selector option to make sure it is working as expected?</t>
+  </si>
+  <si>
+    <t>Card - What are the base asset dimensions necessary for consistency for all card style variations?</t>
+  </si>
+  <si>
+    <t>Alert and Alert Aggregator - We did not cover this in the KT. Can we have documentation on how these components work?</t>
+  </si>
+  <si>
+    <t>How can authors configure button width as a percentage (for example two buttons each taking 50% width on mobile)?</t>
+  </si>
+  <si>
+    <t>How can authors configure buttons to display side-by-side versus stacked, especially across different screen sizes?</t>
+  </si>
+  <si>
+    <t>How can authors override default button colors for campaign-specific designs such as Pinktober or Pride campaigns?</t>
+  </si>
+  <si>
+    <t>How can authors determine the recommended maximum button text length to prevent wrapping or layout issues?</t>
+  </si>
+  <si>
+    <t>How should authors handle long button text or long words so the layout remains consistent across breakpoints?</t>
+  </si>
+  <si>
+    <t>How can authors create responsive button groups without needing custom CSS?</t>
+  </si>
+  <si>
+    <t>How can authors configure a button to trigger a modal linked to an Experience Fragment so that it displays correctly?</t>
+  </si>
+  <si>
+    <t>What is the recommended layout structure for content inside a modal so it appears properly formatted and complete?</t>
+  </si>
+  <si>
+    <t>If modal styling is controlled elsewhere, where should authors configure or adjust modal styling to ensure it looks presentable?</t>
+  </si>
+  <si>
+    <t>What are the recommended guidelines or layout patterns authors should follow when building Experience Fragment content intended for modals?</t>
+  </si>
+  <si>
+    <t>How can authors trigger a modal from a text link instead of only from a button component?</t>
+  </si>
+  <si>
+    <t>How can authors adjust the heading level or visual size of accordion headers without editing HTML directly?</t>
+  </si>
+  <si>
+    <t>When using anchor links there’s no offset and users do NOT get to the right position on the page. when will that be fixed?</t>
+  </si>
+  <si>
+    <t>How can authors determine or define the ID values used for accordion items when creating anchor links?</t>
+  </si>
+  <si>
+    <t>How can authors configure an accordion item to be expanded by default when the page loads, and how many items can be expanded by default?</t>
+  </si>
+  <si>
+    <t>How should accordions be configured when placed on dark background sections?</t>
+  </si>
+  <si>
+    <t>How can authors ensure text and link colors adjust correctly for accessibility when accordions are used on dark backgrounds?</t>
+  </si>
+  <si>
+    <t>What is the this “Simple” layout option for containers, and how should authors use it?</t>
+  </si>
+  <si>
+    <t>When should authors choose this “simple” layout versus a Grid layout for containers?</t>
+  </si>
+  <si>
+    <t>How should authors structure containers so that sections span full width while content remains aligned within the page grid?</t>
+  </si>
+  <si>
+    <t>What is the usage of this Hide Container option, and how should authors ensure hidden content is not indexed or crawled?</t>
+  </si>
+  <si>
+    <t>How can authors properly hide or remove page sections so they are not visible or discoverable by search engines?</t>
+  </si>
+  <si>
+    <t>how do we actually hide/unplubish any component/row/section so that does not get crawled and found?</t>
+  </si>
+  <si>
+    <t>How should authors assign and manage container IDs when they are needed for analytics tracking or personalization?</t>
+  </si>
+  <si>
+    <t>How can teams apply consistent naming conventions for container IDs to ensure they remain readable and standardized?</t>
+  </si>
+  <si>
+    <t>What safeguards or processes should be used to prevent duplicate container IDs across pages?</t>
+  </si>
+  <si>
+    <t>How can authors configure cards so they maintain consistent heights even when card text lengths vary?</t>
+  </si>
+  <si>
+    <t>What settings should authors apply so cards in the same container automatically match height?</t>
+  </si>
+  <si>
+    <t>How should authors configure text truncation for cards, and can it be managed globally instead of individually?</t>
+  </si>
+  <si>
+    <t>How can authors avoid conflicting card styling combinations when selecting card style options?</t>
+  </si>
+  <si>
+    <t>What is the recommended number of cards in a carousel to maintain good usability and performance?</t>
+  </si>
+  <si>
+    <t>How can authors configure a carousel to dynamically pull cards from content sources instead of adding them manually?</t>
+  </si>
+  <si>
+    <t>How should authors manage scheduled or expired cards within a carousel? manual? how do we handle off hours?</t>
+  </si>
+  <si>
+    <t>How can carousel content be shared across multiple layouts such as carousel, grid, or list views using the same data source?</t>
+  </si>
+  <si>
+    <t>How can authors configure the number of cards displayed per device (desktop, tablet, mobile) in a way that works well across screen sizes?</t>
+  </si>
+  <si>
+    <t>How should authors use or configure the Carousel ID, and what purpose does it serve? is it for personalization (Target) or analytics tracking only?</t>
+  </si>
+  <si>
+    <t>How can authors configure query-based content population so grids, lists, or carousels automatically display content based on defined criteria?</t>
+  </si>
+  <si>
+    <t>What criteria can be used in queries to dynamically pull content (tags, folders, templates, metadata, etc.)?</t>
+  </si>
+  <si>
+    <t>How can authors create pages that automatically populate card grids or lists using query rules instead of manual selection?</t>
+  </si>
+  <si>
+    <t>How can authors configure shared content sources so the same query populates multiple layouts such as grid, list, or carousel?</t>
+  </si>
+  <si>
+    <t>How should authors decide when to use the Tabs Cards Filter component versus standard Tabs or filter components?</t>
+  </si>
+  <si>
+    <t>How can authors configure the Tabs Cards Filter component to filter cards using metadata such as tags?</t>
+  </si>
+  <si>
+    <t>How can authors configure the component to pull cards automatically from Experience Fragments or Content Fragments without manually adding each item?</t>
+  </si>
+  <si>
+    <t>How can authors display Experience Fragments dynamically within components such as lists, grids, or carousels?</t>
+  </si>
+  <si>
+    <t>What methods are available to reuse Experience Fragment content across different page layouts?</t>
+  </si>
+  <si>
+    <t>How can authors confirm that the lightbox component supports keyboard navigation and accessibility requirements?</t>
+  </si>
+  <si>
+    <t>How should the lightbox behave for dark mode or accessibility display modes, and how can authors test this behavior?</t>
+  </si>
+  <si>
+    <t>How should authors configure spacer components so spacing displays consistently in author and published views?</t>
+  </si>
+  <si>
+    <t>What is the recommended approach for using spacers inside containers versus outside containers?</t>
+  </si>
+  <si>
+    <t>How should authors apply spacing so duplicate spacers are not required to achieve the intended layout? Or this bug fixed?</t>
+  </si>
+  <si>
+    <t>How can toolbar options within Rich Text Editor components be restricted or simplified for authors?</t>
+  </si>
+  <si>
+    <t>How can administrators restrict certain components (such as Advanced Embed) so they are only available to specific user groups?</t>
+  </si>
+  <si>
+    <t>What are the recommended image specifications (dimensions, aspect ratio, and file size) for container background images?</t>
+  </si>
+  <si>
+    <t>How should authors understand and use template-specific CSS classes, such as those applied in the News page template?</t>
+  </si>
+  <si>
+    <t>What is the recommended page structure for using containers as layout sections, and how should authors organize components within them?</t>
+  </si>
+  <si>
+    <t>In the News page template, what does the applied CSS class actually control and what functionality does it enable?</t>
+  </si>
+  <si>
+    <t>Why does the implementation require placing most components inside containers? Should page sections already act as structural containers by default?</t>
+  </si>
+  <si>
+    <t>What criteria can be used to dynamically pull content (e.g., Experience Fragments, pages, or cards) into components such as carousels, grids, or lists?</t>
+  </si>
+  <si>
+    <t>What query criteria are supported when pulling dynamic content (tags, folders, templates, metadata, etc.)?</t>
+  </si>
+  <si>
+    <t>Can components such as carousels, grids, or lists be configured to pull content dynamically using queries instead of requiring manual selection?</t>
+  </si>
+  <si>
+    <t>How can authors build pages that automatically populate content using query-based lists or card grids rather than manually adding items one by one?</t>
+  </si>
+  <si>
+    <t>Why must authors manually configure the number of cards displayed per device (desktop, tablet, mobile) instead of the component automatically adapting to screen size?</t>
+  </si>
+  <si>
+    <t>Why does the carousel require a Carousel ID, and how is it used?</t>
+  </si>
+  <si>
+    <t>Why are Experience Fragments restricted in how they can be displayed within certain components?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How can we use icons from our own icon library stored in DAM instead of being limited to Font Awesome? </t>
+  </si>
+  <si>
+    <t>If the icon we need is not available in Font Awesome, how should authors add and use custom icons?</t>
+  </si>
+  <si>
+    <t>Are there opportunities to create author presets or templates to reduce the risk of incorrect configuration?</t>
+  </si>
+  <si>
+    <t>What governance exists to ensure authors do not misuse advanced configuration options (CSS classes, embed components, etc.)?</t>
+  </si>
+  <si>
+    <t>How can the platform reduce the need for authors to manually configure responsive behavior?</t>
+  </si>
+  <si>
+    <t>Are components like modals, accordions, and lightboxes fully keyboard accessible?</t>
+  </si>
+  <si>
+    <t>can we add IDs for analytics and target to every component built by vendor?</t>
+  </si>
+  <si>
+    <t>For faq schema how is that enabled and disabled. not al accordions are faqs.</t>
+  </si>
+  <si>
+    <t>Can analytics distinguish between different content sources when the same component is reused across layouts?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1738,6 +2148,14 @@
       <color rgb="FF333333"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1787,10 +2205,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1805,8 +2224,10 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5234,6 +5655,2340 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B5CF2F-573E-C440-96AF-16835B71D151}">
+  <dimension ref="A1:G101"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>554</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>557</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>560</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+    </row>
+    <row r="16" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+    </row>
+    <row r="17" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+    </row>
+    <row r="18" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+    </row>
+    <row r="19" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
+        <v>572</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+    </row>
+    <row r="21" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A21" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+    </row>
+    <row r="22" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A23" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A25" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+    </row>
+    <row r="27" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+    </row>
+    <row r="28" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+    </row>
+    <row r="29" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+    </row>
+    <row r="30" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+    </row>
+    <row r="31" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>582</v>
+      </c>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+    </row>
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+    </row>
+    <row r="34" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+    </row>
+    <row r="35" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>585</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+    </row>
+    <row r="36" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+    </row>
+    <row r="37" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A37" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+    </row>
+    <row r="38" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A38" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A39" s="7" t="s">
+        <v>589</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+    </row>
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+    </row>
+    <row r="41" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+    </row>
+    <row r="42" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A42" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+    </row>
+    <row r="43" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A43" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A44" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+    </row>
+    <row r="45" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A45" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+    </row>
+    <row r="46" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A46" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+    </row>
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+    </row>
+    <row r="48" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A48" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+    </row>
+    <row r="49" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A49" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+    </row>
+    <row r="50" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A50" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+    </row>
+    <row r="51" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A51" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+    </row>
+    <row r="52" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A52" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+    </row>
+    <row r="53" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A53" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+    </row>
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A54" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+    </row>
+    <row r="55" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A55" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+    </row>
+    <row r="56" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A56" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+    </row>
+    <row r="57" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A57" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+    </row>
+    <row r="58" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A58" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+    </row>
+    <row r="59" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A59" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+    </row>
+    <row r="60" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A60" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+    </row>
+    <row r="61" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A61" s="7"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+    </row>
+    <row r="62" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A62" s="7"/>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+    </row>
+    <row r="63" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A63" s="7"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+    </row>
+    <row r="64" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A64" s="7"/>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+    </row>
+    <row r="65" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A65" s="7"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+    </row>
+    <row r="66" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A66" s="7"/>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+    </row>
+    <row r="67" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A67" s="7"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+    </row>
+    <row r="68" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A68" s="7"/>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+    </row>
+    <row r="69" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A69" s="7"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+    </row>
+    <row r="70" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A70" s="7"/>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="7"/>
+      <c r="E70" s="7"/>
+      <c r="F70" s="7"/>
+      <c r="G70" s="7"/>
+    </row>
+    <row r="71" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A71" s="7"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="7"/>
+      <c r="E71" s="7"/>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+    </row>
+    <row r="72" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A72" s="7"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="7"/>
+      <c r="E72" s="7"/>
+      <c r="F72" s="7"/>
+      <c r="G72" s="7"/>
+    </row>
+    <row r="73" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A73" s="7"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+    </row>
+    <row r="74" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A74" s="7"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="7"/>
+      <c r="E74" s="7"/>
+      <c r="F74" s="7"/>
+      <c r="G74" s="7"/>
+    </row>
+    <row r="75" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A75" s="7"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
+      <c r="E75" s="7"/>
+      <c r="F75" s="7"/>
+      <c r="G75" s="7"/>
+    </row>
+    <row r="76" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A76" s="7"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="7"/>
+      <c r="E76" s="7"/>
+      <c r="F76" s="7"/>
+      <c r="G76" s="7"/>
+    </row>
+    <row r="77" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A77" s="7"/>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="7"/>
+      <c r="F77" s="7"/>
+      <c r="G77" s="7"/>
+    </row>
+    <row r="78" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A78" s="7"/>
+      <c r="B78" s="7"/>
+      <c r="C78" s="7"/>
+      <c r="D78" s="7"/>
+      <c r="E78" s="7"/>
+      <c r="F78" s="7"/>
+      <c r="G78" s="7"/>
+    </row>
+    <row r="79" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A79" s="7"/>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7"/>
+      <c r="G79" s="7"/>
+    </row>
+    <row r="80" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A80" s="7"/>
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="7"/>
+      <c r="E80" s="7"/>
+      <c r="F80" s="7"/>
+      <c r="G80" s="7"/>
+    </row>
+    <row r="81" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A81" s="7"/>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="7"/>
+      <c r="E81" s="7"/>
+      <c r="F81" s="7"/>
+      <c r="G81" s="7"/>
+    </row>
+    <row r="82" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A82" s="7"/>
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="7"/>
+      <c r="E82" s="7"/>
+      <c r="F82" s="7"/>
+      <c r="G82" s="7"/>
+    </row>
+    <row r="83" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A83" s="7"/>
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7"/>
+      <c r="G83" s="7"/>
+    </row>
+    <row r="84" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A84" s="7"/>
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+      <c r="D84" s="7"/>
+      <c r="E84" s="7"/>
+      <c r="F84" s="7"/>
+      <c r="G84" s="7"/>
+    </row>
+    <row r="85" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A85" s="7"/>
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="7"/>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="7"/>
+    </row>
+    <row r="86" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A86" s="7"/>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="7"/>
+      <c r="E86" s="7"/>
+      <c r="F86" s="7"/>
+      <c r="G86" s="7"/>
+    </row>
+    <row r="87" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A87" s="7"/>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="7"/>
+      <c r="E87" s="7"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="7"/>
+    </row>
+    <row r="88" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A88" s="7"/>
+      <c r="B88" s="7"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="7"/>
+      <c r="E88" s="7"/>
+      <c r="F88" s="7"/>
+      <c r="G88" s="7"/>
+    </row>
+    <row r="89" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A89" s="7"/>
+      <c r="B89" s="7"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="7"/>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7"/>
+      <c r="G89" s="7"/>
+    </row>
+    <row r="90" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A90" s="7"/>
+      <c r="B90" s="7"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="7"/>
+      <c r="E90" s="7"/>
+      <c r="F90" s="7"/>
+      <c r="G90" s="7"/>
+    </row>
+    <row r="91" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A91" s="7"/>
+      <c r="B91" s="7"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="7"/>
+      <c r="E91" s="7"/>
+      <c r="F91" s="7"/>
+      <c r="G91" s="7"/>
+    </row>
+    <row r="92" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A92" s="7"/>
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="7"/>
+      <c r="E92" s="7"/>
+      <c r="F92" s="7"/>
+      <c r="G92" s="7"/>
+    </row>
+    <row r="93" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A93" s="7"/>
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="7"/>
+      <c r="E93" s="7"/>
+      <c r="F93" s="7"/>
+      <c r="G93" s="7"/>
+    </row>
+    <row r="94" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A94" s="7"/>
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="7"/>
+      <c r="E94" s="7"/>
+      <c r="F94" s="7"/>
+      <c r="G94" s="7"/>
+    </row>
+    <row r="95" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A95" s="7"/>
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="7"/>
+      <c r="E95" s="7"/>
+      <c r="F95" s="7"/>
+      <c r="G95" s="7"/>
+    </row>
+    <row r="96" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A96" s="7"/>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="7"/>
+      <c r="E96" s="7"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="7"/>
+    </row>
+    <row r="97" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A97" s="7"/>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="7"/>
+      <c r="E97" s="7"/>
+      <c r="F97" s="7"/>
+      <c r="G97" s="7"/>
+    </row>
+    <row r="98" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A98" s="7"/>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="7"/>
+      <c r="E98" s="7"/>
+      <c r="F98" s="7"/>
+      <c r="G98" s="7"/>
+    </row>
+    <row r="99" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A99" s="7"/>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="7"/>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7"/>
+      <c r="G99" s="7"/>
+    </row>
+    <row r="100" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A100" s="7"/>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="7"/>
+      <c r="E100" s="7"/>
+      <c r="F100" s="7"/>
+      <c r="G100" s="7"/>
+    </row>
+    <row r="101" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A101" s="7"/>
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="7"/>
+      <c r="E101" s="7"/>
+      <c r="F101" s="7"/>
+      <c r="G101" s="7"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A10" r:id="rId1" display="https://shrss.atlassian.net/wiki/spaces/AA/pages/edit-v2/4386291724" xr:uid="{902AE73C-C708-8147-B3A1-F5311726DCBC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D226C679-6118-7C44-8F83-90D563480629}">
+  <dimension ref="A1:G102"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>610</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>620</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>623</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+    </row>
+    <row r="16" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+    </row>
+    <row r="17" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+    </row>
+    <row r="18" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+    </row>
+    <row r="19" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+    </row>
+    <row r="21" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A21" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+    </row>
+    <row r="22" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A23" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A25" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+    </row>
+    <row r="27" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+    </row>
+    <row r="28" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+    </row>
+    <row r="29" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+    </row>
+    <row r="30" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>638</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+    </row>
+    <row r="31" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+    </row>
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+    </row>
+    <row r="34" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+    </row>
+    <row r="35" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>643</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+    </row>
+    <row r="36" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+    </row>
+    <row r="37" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A37" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+    </row>
+    <row r="38" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A38" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A39" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+    </row>
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+    </row>
+    <row r="41" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+    </row>
+    <row r="42" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A42" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+    </row>
+    <row r="43" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A43" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A44" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+    </row>
+    <row r="45" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A45" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+    </row>
+    <row r="46" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A46" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+    </row>
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+    </row>
+    <row r="48" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A48" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+    </row>
+    <row r="49" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A49" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+    </row>
+    <row r="50" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A50" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+    </row>
+    <row r="51" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A51" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+    </row>
+    <row r="52" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A52" s="7" t="s">
+        <v>660</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+    </row>
+    <row r="53" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A53" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+    </row>
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A54" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+    </row>
+    <row r="55" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A55" s="7" t="s">
+        <v>663</v>
+      </c>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+    </row>
+    <row r="56" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A56" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+    </row>
+    <row r="57" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A57" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+    </row>
+    <row r="58" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A58" s="7" t="s">
+        <v>666</v>
+      </c>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+    </row>
+    <row r="59" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A59" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+    </row>
+    <row r="60" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A60" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+    </row>
+    <row r="61" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A61" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+    </row>
+    <row r="62" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A62" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+    </row>
+    <row r="63" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A63" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+    </row>
+    <row r="64" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A64" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+    </row>
+    <row r="65" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A65" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+    </row>
+    <row r="66" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A66" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+    </row>
+    <row r="67" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A67" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+    </row>
+    <row r="68" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A68" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+    </row>
+    <row r="69" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A69" s="7" t="s">
+        <v>676</v>
+      </c>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+    </row>
+    <row r="70" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A70" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="7"/>
+      <c r="E70" s="7"/>
+      <c r="F70" s="7"/>
+      <c r="G70" s="7"/>
+    </row>
+    <row r="71" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A71" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="7"/>
+      <c r="E71" s="7"/>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+    </row>
+    <row r="72" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A72" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="7"/>
+      <c r="E72" s="7"/>
+      <c r="F72" s="7"/>
+      <c r="G72" s="7"/>
+    </row>
+    <row r="73" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A73" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+    </row>
+    <row r="74" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A74" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="7"/>
+      <c r="E74" s="7"/>
+      <c r="F74" s="7"/>
+      <c r="G74" s="7"/>
+    </row>
+    <row r="75" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A75" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
+      <c r="E75" s="7"/>
+      <c r="F75" s="7"/>
+      <c r="G75" s="7"/>
+    </row>
+    <row r="76" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A76" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="7"/>
+      <c r="E76" s="7"/>
+      <c r="F76" s="7"/>
+      <c r="G76" s="7"/>
+    </row>
+    <row r="77" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A77" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="7"/>
+      <c r="F77" s="7"/>
+      <c r="G77" s="7"/>
+    </row>
+    <row r="78" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A78" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="B78" s="7"/>
+      <c r="C78" s="7"/>
+      <c r="D78" s="7"/>
+      <c r="E78" s="7"/>
+      <c r="F78" s="7"/>
+      <c r="G78" s="7"/>
+    </row>
+    <row r="79" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A79" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7"/>
+      <c r="G79" s="7"/>
+    </row>
+    <row r="80" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A80" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="7"/>
+      <c r="E80" s="7"/>
+      <c r="F80" s="7"/>
+      <c r="G80" s="7"/>
+    </row>
+    <row r="81" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A81" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="7"/>
+      <c r="E81" s="7"/>
+      <c r="F81" s="7"/>
+      <c r="G81" s="7"/>
+    </row>
+    <row r="82" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A82" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="7"/>
+      <c r="E82" s="7"/>
+      <c r="F82" s="7"/>
+      <c r="G82" s="7"/>
+    </row>
+    <row r="83" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A83" s="7"/>
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7"/>
+      <c r="G83" s="7"/>
+    </row>
+    <row r="84" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A84" s="7"/>
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+      <c r="D84" s="7"/>
+      <c r="E84" s="7"/>
+      <c r="F84" s="7"/>
+      <c r="G84" s="7"/>
+    </row>
+    <row r="85" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A85" s="7"/>
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="7"/>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="7"/>
+    </row>
+    <row r="86" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A86" s="7"/>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="7"/>
+      <c r="E86" s="7"/>
+      <c r="F86" s="7"/>
+      <c r="G86" s="7"/>
+    </row>
+    <row r="87" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A87" s="7"/>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="7"/>
+      <c r="E87" s="7"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="7"/>
+    </row>
+    <row r="88" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A88" s="7"/>
+      <c r="B88" s="7"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="7"/>
+      <c r="E88" s="7"/>
+      <c r="F88" s="7"/>
+      <c r="G88" s="7"/>
+    </row>
+    <row r="89" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A89" s="7"/>
+      <c r="B89" s="7"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="7"/>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7"/>
+      <c r="G89" s="7"/>
+    </row>
+    <row r="90" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A90" s="7"/>
+      <c r="B90" s="7"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="7"/>
+      <c r="E90" s="7"/>
+      <c r="F90" s="7"/>
+      <c r="G90" s="7"/>
+    </row>
+    <row r="91" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A91" s="7"/>
+      <c r="B91" s="7"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="7"/>
+      <c r="E91" s="7"/>
+      <c r="F91" s="7"/>
+      <c r="G91" s="7"/>
+    </row>
+    <row r="92" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A92" s="7"/>
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="7"/>
+      <c r="E92" s="7"/>
+      <c r="F92" s="7"/>
+      <c r="G92" s="7"/>
+    </row>
+    <row r="93" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A93" s="7"/>
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="7"/>
+      <c r="E93" s="7"/>
+      <c r="F93" s="7"/>
+      <c r="G93" s="7"/>
+    </row>
+    <row r="94" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A94" s="7"/>
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="7"/>
+      <c r="E94" s="7"/>
+      <c r="F94" s="7"/>
+      <c r="G94" s="7"/>
+    </row>
+    <row r="95" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A95" s="7"/>
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="7"/>
+      <c r="E95" s="7"/>
+      <c r="F95" s="7"/>
+      <c r="G95" s="7"/>
+    </row>
+    <row r="96" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A96" s="7"/>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="7"/>
+      <c r="E96" s="7"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="7"/>
+    </row>
+    <row r="97" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A97" s="7"/>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="7"/>
+      <c r="E97" s="7"/>
+      <c r="F97" s="7"/>
+      <c r="G97" s="7"/>
+    </row>
+    <row r="98" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A98" s="7"/>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="7"/>
+      <c r="E98" s="7"/>
+      <c r="F98" s="7"/>
+      <c r="G98" s="7"/>
+    </row>
+    <row r="99" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A99" s="7"/>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="7"/>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7"/>
+      <c r="G99" s="7"/>
+    </row>
+    <row r="100" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A100" s="7"/>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="7"/>
+      <c r="E100" s="7"/>
+      <c r="F100" s="7"/>
+      <c r="G100" s="7"/>
+    </row>
+    <row r="101" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A101" s="7"/>
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="7"/>
+      <c r="E101" s="7"/>
+      <c r="F101" s="7"/>
+      <c r="G101" s="7"/>
+    </row>
+    <row r="102" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A102" s="7"/>
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="7"/>
+      <c r="E102" s="7"/>
+      <c r="F102" s="7"/>
+      <c r="G102" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H29"/>

</xml_diff>